<commit_message>
deploy: 2026-09-10 15:02 (from f2a1e3a)
</commit_message>
<xml_diff>
--- a/templates/TEMPLATE_หน้าตัดอลูมิเนียม.xlsx
+++ b/templates/TEMPLATE_หน้าตัดอลูมิเนียม.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -414,6 +414,15 @@
       <c r="C3" t="str">
         <v>ความยาวมาตรฐาน (เมตร)</v>
       </c>
+      <c r="D3" t="str">
+        <v>กลุ่มหน้าตัด</v>
+      </c>
+      <c r="E3" t="str">
+        <v>รุ่น/ซีรีส์</v>
+      </c>
+      <c r="F3" t="str">
+        <v>ความหนา (มม.)</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -425,10 +434,19 @@
       <c r="C4" t="str">
         <v>เช่น 6.4 (เว้นว่างได้ ค่าเริ่มต้น 6.4)</v>
       </c>
+      <c r="D4" t="str">
+        <v>เช่น กล่องร่อง (สำหรับผูกกับ BOM Template)</v>
+      </c>
+      <c r="E4" t="str">
+        <v>เช่น ทั่วไป, ยูโร, วิสดอม</v>
+      </c>
+      <c r="F4" t="str">
+        <v>เช่น 1.2</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>